<commit_message>
add essen (zip 45127) weather files
</commit_message>
<xml_diff>
--- a/districtgenerator/data/plz_geocoord_matched.xlsx
+++ b/districtgenerator/data/plz_geocoord_matched.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Script\districtgenerator\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dokumente\Daten\Git\Programmieren\districtgenerator\districtgenerator\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EBE6AF8-3107-4006-A186-E36207B9ACE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C118852-8D21-4E88-A296-444873D0728D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-5325" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>PLZ</t>
   </si>
@@ -71,13 +72,16 @@
   </si>
   <si>
     <t>TRY2015_507755060854_Jahr.dat</t>
+  </si>
+  <si>
+    <t>TRY2015_514636069818_Jahr.dat</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -89,6 +93,12 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -137,7 +147,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -147,6 +157,9 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -449,13 +462,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="4" max="4" width="39" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -475,7 +490,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6">
       <c r="A2" s="4">
         <v>44137</v>
       </c>
@@ -495,7 +510,7 @@
         <v>13.71674948054328</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6">
       <c r="A3" s="3">
         <v>50667</v>
       </c>
@@ -515,7 +530,7 @@
         <v>13.74475915535144</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6">
       <c r="A4" s="3">
         <v>52064</v>
       </c>
@@ -535,7 +550,7 @@
         <v>13.73224853694335</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6">
       <c r="A5" s="3">
         <v>34117</v>
       </c>
@@ -555,7 +570,7 @@
         <v>13.80754694289841</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6">
       <c r="A6" s="3">
         <v>10115</v>
       </c>
@@ -575,7 +590,7 @@
         <v>13.797341617316221</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6">
       <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
@@ -595,7 +610,7 @@
         <v>13.7212110431462</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6">
       <c r="A8" s="3">
         <v>80331</v>
       </c>
@@ -615,7 +630,7 @@
         <v>13.718235479892741</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6">
       <c r="A9" s="3">
         <v>20354</v>
       </c>
@@ -635,7 +650,7 @@
         <v>13.71972266695261</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6">
       <c r="A10" s="3">
         <v>79100</v>
       </c>
@@ -655,7 +670,7 @@
         <v>13.68797903256106</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6">
       <c r="A11" s="3">
         <v>38100</v>
       </c>
@@ -674,6 +689,17 @@
       <c r="F11">
         <v>13.629674415765569</v>
       </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="3">
+        <v>45127</v>
+      </c>
+      <c r="D12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="D16" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>